<commit_message>
inclusão da coluna tempo de inferencia
</commit_message>
<xml_diff>
--- a/tabelas/tabelas.xlsx
+++ b/tabelas/tabelas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/53f471b9ff959fbc/Documents/0_BSI/0TCC/Resultados/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\TCC\tabelas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{10622787-AA72-4202-8C16-06986B635F74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50A65BEA-45D3-4965-A25E-7DD329229E36}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD3F23D0-937B-4288-B117-6F11277661CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24210" yWindow="3345" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="6" xr2:uid="{13F06048-EB8B-4FDA-AF69-07DBD3E39C1E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="6" xr2:uid="{13F06048-EB8B-4FDA-AF69-07DBD3E39C1E}"/>
   </bookViews>
   <sheets>
     <sheet name="LeNet" sheetId="1" r:id="rId1"/>
@@ -19,8 +19,7 @@
     <sheet name="GoogLeNet" sheetId="4" r:id="rId4"/>
     <sheet name="MobileNet" sheetId="5" r:id="rId5"/>
     <sheet name="Inferencia" sheetId="6" r:id="rId6"/>
-    <sheet name="EficienciaCusto" sheetId="7" r:id="rId7"/>
-    <sheet name="Planilha1" sheetId="8" r:id="rId8"/>
+    <sheet name="EficienciaCusto" sheetId="8" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="38">
   <si>
     <t>Modelo</t>
   </si>
@@ -129,9 +128,6 @@
     <t>Lenet-5</t>
   </si>
   <si>
-    <t>Eficiência e Custo Computacional</t>
-  </si>
-  <si>
     <t>Modelos</t>
   </si>
   <si>
@@ -151,6 +147,15 @@
   </si>
   <si>
     <t>Desempenho X Eficiência</t>
+  </si>
+  <si>
+    <t>Tempo de Inferência</t>
+  </si>
+  <si>
+    <t>Média</t>
+  </si>
+  <si>
+    <t>Desvio Padrão</t>
   </si>
 </sst>
 </file>
@@ -224,50 +229,9 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="43">
+  <dxfs count="36">
     <dxf>
       <numFmt numFmtId="164" formatCode="0.00000"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.00000"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.00000"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -430,10 +394,10 @@
   <autoFilter ref="B5:F17" xr:uid="{42A7CCED-0E68-45DF-9CBC-9E670B1486C0}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{CB903ED8-FC88-43B5-A04E-C414D1B9CB62}" name="Modelo"/>
-    <tableColumn id="2" xr3:uid="{4B634E77-212D-4997-BA43-943EDA37543D}" name="Perda Treino" dataDxfId="42"/>
-    <tableColumn id="3" xr3:uid="{92859825-22E3-4FA9-9C1D-F02E29E0D44B}" name="Acurácia Treino" dataDxfId="41"/>
-    <tableColumn id="4" xr3:uid="{57583B4E-F0CD-4677-B970-CF6215DAA331}" name="Perda Validação" dataDxfId="40"/>
-    <tableColumn id="5" xr3:uid="{0E1E3B98-2262-4CCB-8164-E077F47D133B}" name="Acurácia Validação" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{4B634E77-212D-4997-BA43-943EDA37543D}" name="Perda Treino" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{92859825-22E3-4FA9-9C1D-F02E29E0D44B}" name="Acurácia Treino" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{57583B4E-F0CD-4677-B970-CF6215DAA331}" name="Perda Validação" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{0E1E3B98-2262-4CCB-8164-E077F47D133B}" name="Acurácia Validação" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -444,10 +408,10 @@
   <autoFilter ref="B4:F16" xr:uid="{0672EF86-9B43-43F6-A288-74C94587B6CD}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{A812A20D-EB45-4072-B3FF-DF34AC513729}" name="Modelo"/>
-    <tableColumn id="2" xr3:uid="{AC25AC79-F200-4561-BF29-BEE5F767B72E}" name="Perda Treino" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{057CD4D6-D043-47D0-96D2-CFDC9F6F6E98}" name="Acurácia Treino" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{1C3DFBE2-C68D-4D3C-9F71-FA116D772A6D}" name="Perda Validação" dataDxfId="36"/>
-    <tableColumn id="5" xr3:uid="{687ABCC5-40D9-4495-85D0-2DC1E226E6EC}" name="Acurácia Validação" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{AC25AC79-F200-4561-BF29-BEE5F767B72E}" name="Perda Treino" dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{057CD4D6-D043-47D0-96D2-CFDC9F6F6E98}" name="Acurácia Treino" dataDxfId="30"/>
+    <tableColumn id="4" xr3:uid="{1C3DFBE2-C68D-4D3C-9F71-FA116D772A6D}" name="Perda Validação" dataDxfId="29"/>
+    <tableColumn id="5" xr3:uid="{687ABCC5-40D9-4495-85D0-2DC1E226E6EC}" name="Acurácia Validação" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -458,10 +422,10 @@
   <autoFilter ref="B4:F16" xr:uid="{D6AA89FA-8130-4D2F-9900-384E26D5A570}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{D4F8D0C9-A7F1-4ADC-A78C-FFE8CF1FBBC7}" name="Modelo"/>
-    <tableColumn id="2" xr3:uid="{17C97566-AE62-4FD3-B098-073FE84D6763}" name="Perda Treino" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{FD7DE413-454E-4236-B597-8A7B825BFB4A}" name="Acurácia Treino" dataDxfId="33"/>
-    <tableColumn id="4" xr3:uid="{8852E415-56FB-40CA-9C65-6DC604729AA3}" name="Perda Validação" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{ABF7EDC7-2C73-4524-8802-9735A734BA53}" name="Acurácia Validação" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{17C97566-AE62-4FD3-B098-073FE84D6763}" name="Perda Treino" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{FD7DE413-454E-4236-B597-8A7B825BFB4A}" name="Acurácia Treino" dataDxfId="26"/>
+    <tableColumn id="4" xr3:uid="{8852E415-56FB-40CA-9C65-6DC604729AA3}" name="Perda Validação" dataDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{ABF7EDC7-2C73-4524-8802-9735A734BA53}" name="Acurácia Validação" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -472,10 +436,10 @@
   <autoFilter ref="B4:F16" xr:uid="{002431A3-C699-47A2-88EB-D3DECA80E7A4}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{2B47B00D-562F-44D2-AE18-F89A8ED96A0D}" name="Modelo"/>
-    <tableColumn id="2" xr3:uid="{0F9F9B52-F2C3-49F0-8C14-0D67638B7AC5}" name="Perda Treino" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{37B0C17F-4682-48D4-AF89-06E13239802A}" name="Acurácia Treino" dataDxfId="29"/>
-    <tableColumn id="4" xr3:uid="{D58038CB-FF6B-4886-960C-39868883D8F2}" name="Perda Validação" dataDxfId="28"/>
-    <tableColumn id="5" xr3:uid="{1E7BFA72-CB3D-46ED-A30A-A0FD0940062E}" name="Acurácia Validação" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{0F9F9B52-F2C3-49F0-8C14-0D67638B7AC5}" name="Perda Treino" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{37B0C17F-4682-48D4-AF89-06E13239802A}" name="Acurácia Treino" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{D58038CB-FF6B-4886-960C-39868883D8F2}" name="Perda Validação" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{1E7BFA72-CB3D-46ED-A30A-A0FD0940062E}" name="Acurácia Validação" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -486,54 +450,40 @@
   <autoFilter ref="B4:F16" xr:uid="{B31703F6-ACEB-43F3-A4F3-B540607AD1FB}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{0EA81A56-C530-41C7-985B-C19780CAA2C3}" name="Modelo"/>
-    <tableColumn id="2" xr3:uid="{EB87C832-2BB9-4819-A7AF-CE9047FFAE0A}" name="Perda Treino" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{48A4ACAC-615B-4687-95AD-E08AE8B13597}" name="Acurácia Treino" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{040E087B-3367-42B3-8841-F475B7E4E7D2}" name="Perda Validação" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{539F3614-D2C6-4283-BA24-B18B50EB207E}" name="Acurácia Validação" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{EB87C832-2BB9-4819-A7AF-CE9047FFAE0A}" name="Perda Treino" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{48A4ACAC-615B-4687-95AD-E08AE8B13597}" name="Acurácia Treino" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{040E087B-3367-42B3-8841-F475B7E4E7D2}" name="Perda Validação" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{539F3614-D2C6-4283-BA24-B18B50EB207E}" name="Acurácia Validação" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{BC6BD6A3-AC2C-4B1E-9335-88825FD062A9}" name="Tabela8" displayName="Tabela8" ref="B3:F8" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{BC6BD6A3-AC2C-4B1E-9335-88825FD062A9}" name="Tabela8" displayName="Tabela8" ref="B3:F8" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
   <autoFilter ref="B3:F8" xr:uid="{BC6BD6A3-AC2C-4B1E-9335-88825FD062A9}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{70E6298B-0460-4437-862E-E64C6576E345}" name="Melhor Modelo" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{8116BC02-003C-4DD0-B9F9-245028FEAB54}" name="Acurácia" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{76F274EF-0A7A-4F8D-9066-F105B3DE71AD}" name="Precisão" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{DBA3BE60-6C8A-4C1A-8BF9-A77FDFE82F3D}" name="Revocação" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{14DC8645-FD70-41F2-A667-A0F896372849}" name="Medida-F1" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{70E6298B-0460-4437-862E-E64C6576E345}" name="Melhor Modelo" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{8116BC02-003C-4DD0-B9F9-245028FEAB54}" name="Acurácia" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{76F274EF-0A7A-4F8D-9066-F105B3DE71AD}" name="Precisão" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{DBA3BE60-6C8A-4C1A-8BF9-A77FDFE82F3D}" name="Revocação" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{14DC8645-FD70-41F2-A667-A0F896372849}" name="Medida-F1" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9C6E1CC4-4A0F-4914-80C2-ECBFEDF614F1}" name="Tabela9" displayName="Tabela9" ref="B5:G10" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
-  <autoFilter ref="B5:G10" xr:uid="{9C6E1CC4-4A0F-4914-80C2-ECBFEDF614F1}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{13CAA92D-0FBB-40CC-BB20-150EBDF0A3C4}" name="Modelos" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{9A5847B4-157E-49AC-845B-C252AD108487}" name="Emissão de carbono" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{A5686EC6-3DE7-4E33-B23A-7365E55DF881}" name="Consumo de Energia" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{1EDCC311-D1E1-4A9E-BD9B-A56C3B09D34D}" name="Número de Parâmetros" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{6F55AF8E-E4AE-4C39-A831-BB9E4D6B5411}" name="FLOPs" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{23278518-3B39-44EC-B094-FC97E7A04851}" name="Tempo de treino" dataDxfId="8"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E253A832-1C69-4A1E-8DF2-31DE7F233415}" name="Tabela94" displayName="Tabela94" ref="B5:G10" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
-  <autoFilter ref="B5:G10" xr:uid="{E253A832-1C69-4A1E-8DF2-31DE7F233415}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B4A77944-374E-4B7A-93C2-C687F79C9092}" name="Modelos" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{85191E0C-97BD-45DF-9E4E-CA2193D04180}" name="Emissão de carbono" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{9EA077B6-C438-4876-8B6D-198EF4D5BF19}" name="Consumo de Energia" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{893E4838-4497-44B8-8F78-0D712B0B5248}" name="Número de Parâmetros" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{71535624-8785-4CB5-8FF5-CF18CD385372}" name="FLOPs" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{047AC4F3-AC89-403A-A6DA-7CE3EC6A4F86}" name="Tempo de treino" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E253A832-1C69-4A1E-8DF2-31DE7F233415}" name="Tabela94" displayName="Tabela94" ref="B5:H12" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="B5:H12" xr:uid="{E253A832-1C69-4A1E-8DF2-31DE7F233415}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{B4A77944-374E-4B7A-93C2-C687F79C9092}" name="Modelos" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{85191E0C-97BD-45DF-9E4E-CA2193D04180}" name="Emissão de carbono" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{9EA077B6-C438-4876-8B6D-198EF4D5BF19}" name="Consumo de Energia" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{893E4838-4497-44B8-8F78-0D712B0B5248}" name="Número de Parâmetros" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{71535624-8785-4CB5-8FF5-CF18CD385372}" name="FLOPs" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{047AC4F3-AC89-403A-A6DA-7CE3EC6A4F86}" name="Tempo de treino" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{BDE67346-2B24-4B79-B8FC-6620E2C450DB}" name="Tempo de Inferência" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2255,44 +2205,48 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46D5B12F-18D1-49B7-B270-772A26772B29}">
-  <dimension ref="B3:G10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8802D625-7BED-4003-92FF-7A504D813763}">
+  <dimension ref="B3:H12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10.85546875" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="21.140625" customWidth="1"/>
     <col min="4" max="4" width="21.7109375" customWidth="1"/>
     <col min="5" max="5" width="23.85546875" customWidth="1"/>
     <col min="6" max="6" width="15.140625" customWidth="1"/>
     <col min="7" max="7" width="17.85546875" customWidth="1"/>
+    <col min="8" max="8" width="22.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B5" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="5" spans="2:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="H5" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
         <v>27</v>
       </c>
@@ -2311,8 +2265,11 @@
       <c r="G6" s="7">
         <v>132.05211</v>
       </c>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="H6" s="7">
+        <v>1.1288937999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
         <v>18</v>
       </c>
@@ -2331,8 +2288,11 @@
       <c r="G7" s="7">
         <v>546.07587999999998</v>
       </c>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="H7" s="7">
+        <v>1.6999272000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
         <v>19</v>
       </c>
@@ -2351,8 +2311,11 @@
       <c r="G8" s="7">
         <v>667.21659999999997</v>
       </c>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="H8" s="7">
+        <v>2.1356771999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
         <v>20</v>
       </c>
@@ -2371,8 +2334,11 @@
       <c r="G9" s="7">
         <v>626.06713999999999</v>
       </c>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="H9" s="7">
+        <v>1.8502673000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>21</v>
       </c>
@@ -2391,151 +2357,66 @@
       <c r="G10" s="7">
         <v>424.10750999999999</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8802D625-7BED-4003-92FF-7A504D813763}">
-  <dimension ref="B3:G10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="10.85546875" customWidth="1"/>
-    <col min="3" max="3" width="21.140625" customWidth="1"/>
-    <col min="4" max="4" width="21.7109375" customWidth="1"/>
-    <col min="5" max="5" width="23.85546875" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" customWidth="1"/>
-    <col min="7" max="7" width="17.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B5" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="7">
-        <v>0.93286000000000002</v>
-      </c>
-      <c r="D6" s="7">
-        <v>49.604089999999999</v>
-      </c>
-      <c r="E6" s="6">
-        <v>609354</v>
-      </c>
-      <c r="F6" s="6">
-        <v>11401984</v>
-      </c>
-      <c r="G6" s="7">
-        <v>132.05211</v>
-      </c>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="7">
-        <v>6.3491</v>
-      </c>
-      <c r="D7" s="7">
-        <v>95.363370000000003</v>
-      </c>
-      <c r="E7" s="6">
-        <v>23271114</v>
-      </c>
-      <c r="F7" s="6">
-        <v>147910912</v>
-      </c>
-      <c r="G7" s="7">
-        <v>546.07587999999998</v>
-      </c>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="7">
-        <v>6.4630000000000001</v>
-      </c>
-      <c r="D8" s="7">
-        <v>87.374949999999998</v>
-      </c>
-      <c r="E8" s="6">
-        <v>21292042</v>
-      </c>
-      <c r="F8" s="6">
-        <v>69921536</v>
-      </c>
-      <c r="G8" s="7">
-        <v>667.21659999999997</v>
-      </c>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B9" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" s="7">
-        <v>4.3731999999999998</v>
-      </c>
-      <c r="D9" s="7">
-        <v>75.870549999999994</v>
-      </c>
-      <c r="E9" s="6">
-        <v>5977530</v>
-      </c>
-      <c r="F9" s="6">
-        <v>36235520</v>
-      </c>
-      <c r="G9" s="7">
-        <v>626.06713999999999</v>
-      </c>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B10" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="7">
-        <v>1.46991</v>
-      </c>
-      <c r="D10" s="7">
-        <v>66.016260000000003</v>
-      </c>
-      <c r="E10" s="6">
-        <v>24618</v>
-      </c>
-      <c r="F10" s="6">
-        <v>8054656</v>
-      </c>
-      <c r="G10" s="7">
-        <v>424.10750999999999</v>
+      <c r="H10" s="7">
+        <v>1.2544276000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B11" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="7">
+        <f>AVERAGE(C6:C10)</f>
+        <v>3.9176139999999995</v>
+      </c>
+      <c r="D11" s="7">
+        <f t="shared" ref="D11:H11" si="0">AVERAGE(D6:D10)</f>
+        <v>74.845844</v>
+      </c>
+      <c r="E11" s="6">
+        <f t="shared" si="0"/>
+        <v>10234931.6</v>
+      </c>
+      <c r="F11" s="6">
+        <f t="shared" si="0"/>
+        <v>54704921.600000001</v>
+      </c>
+      <c r="G11" s="7">
+        <f t="shared" si="0"/>
+        <v>479.10384799999991</v>
+      </c>
+      <c r="H11" s="7">
+        <f t="shared" si="0"/>
+        <v>1.6138386199999999</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B12" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="7">
+        <f>STDEV(C6:C10)</f>
+        <v>2.6219593805358619</v>
+      </c>
+      <c r="D12" s="7">
+        <f t="shared" ref="D12:H12" si="1">STDEV(D6:D10)</f>
+        <v>17.986836098352036</v>
+      </c>
+      <c r="E12" s="6">
+        <f t="shared" si="1"/>
+        <v>11260877.61113124</v>
+      </c>
+      <c r="F12" s="6">
+        <f t="shared" si="1"/>
+        <v>57687547.358691938</v>
+      </c>
+      <c r="G12" s="7">
+        <f t="shared" si="1"/>
+        <v>215.02289167256757</v>
+      </c>
+      <c r="H12" s="7">
+        <f t="shared" si="1"/>
+        <v>0.41832195365879615</v>
       </c>
     </row>
   </sheetData>

</xml_diff>